<commit_message>
Convert IST to single-assay schema
</commit_message>
<xml_diff>
--- a/illumina-spatial-v0/latest/illumina-spatial-v0.xlsx
+++ b/illumina-spatial-v0/latest/illumina-spatial-v0.xlsx
@@ -8,15 +8,21 @@
   <sheets>
     <sheet name="Illumina Spatial v0" r:id="rId3" sheetId="1"/>
     <sheet name="dataset_type" r:id="rId4" sheetId="2"/>
-    <sheet name="mapped_area_unit" r:id="rId5" sheetId="3"/>
-    <sheet name="capture_area_id" r:id="rId6" sheetId="4"/>
-    <sheet name="capture_area_width_unit" r:id="rId7" sheetId="5"/>
-    <sheet name="capture_area_height_unit" r:id="rId8" sheetId="6"/>
-    <sheet name="permeabilization_time_unit" r:id="rId9" sheetId="7"/>
-    <sheet name="preparation_instrument_vendor" r:id="rId10" sheetId="8"/>
-    <sheet name="preparation_instrument_model" r:id="rId11" sheetId="9"/>
-    <sheet name="spatial_discreatization_method" r:id="rId12" sheetId="10"/>
-    <sheet name=".metadata" r:id="rId13" sheetId="11"/>
+    <sheet name="analyte_class" r:id="rId5" sheetId="3"/>
+    <sheet name="is_targeted" r:id="rId6" sheetId="4"/>
+    <sheet name="acquisition_instrument_vendor" r:id="rId7" sheetId="5"/>
+    <sheet name="acquisition_instrument_model" r:id="rId8" sheetId="6"/>
+    <sheet name="source_storage_duration_unit" r:id="rId9" sheetId="7"/>
+    <sheet name="time_since_acquisition_instrume" r:id="rId10" sheetId="8"/>
+    <sheet name="mapped_area_unit" r:id="rId11" sheetId="9"/>
+    <sheet name="capture_area_id" r:id="rId12" sheetId="10"/>
+    <sheet name="capture_area_width_unit" r:id="rId13" sheetId="11"/>
+    <sheet name="capture_area_height_unit" r:id="rId14" sheetId="12"/>
+    <sheet name="permeabilization_time_unit" r:id="rId15" sheetId="13"/>
+    <sheet name="preparation_instrument_vendor" r:id="rId16" sheetId="14"/>
+    <sheet name="preparation_instrument_model" r:id="rId17" sheetId="15"/>
+    <sheet name="spatial_discreatization_method" r:id="rId18" sheetId="16"/>
+    <sheet name=".metadata" r:id="rId19" sheetId="17"/>
   </sheets>
 </workbook>
 </file>
@@ -58,16 +64,75 @@
     </comment>
     <comment ref="D1" authorId="1">
       <text>
-        <t>The specific type of dataset being produced. Example: RNAseq</t>
+        <t>(Required) The specific type of dataset being produced. Example: RNAseq</t>
       </text>
     </comment>
     <comment ref="E1" authorId="1">
+      <text>
+        <t>(Required) The analyte class which is the target molecule that the assay is
+measuring. Example: DNA</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="1">
+      <text>
+        <t>(Required) Indicates whether a specific molecule or set of molecules is targeted
+for detection or measurement by the assay. Example: Yes</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="1">
+      <text>
+        <t>(Required) The company that manufactures or supplies the acquisition instrument.
+An acquisition instrument is a device equipped with signal detection hardware
+and signal processing software. It captures signals produced by assays, such as
+variations in light intensity or color, or signals corresponding to molecular
+mass. If the instrument was custom-built or developed internally, enter
+"In-House". Example: Illumina</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="1">
+      <text>
+        <t>(Required) The specific model of the acquisition instrument, as manufacturers
+often offer various versions with differing features or sensitivities. These
+differences may be relevant to the processing or interpretation of the data. If
+the instrument was custom-built or developed internally, enter "In-House". If
+the model is unknown, enter "Unknown". Example: HiSeq 4000</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="1">
+      <text>
+        <t>(Required) The length of time the sample was stored prior to processing it. For
+assays performed on tissue sections, this refers to how long the tissue section
+(e.g., slide) was stored before the assay began (e.g., imaging). For assays
+performed on suspensions, such as sequencing, it refers to how long the
+suspension was stored before library construction started. Example: 12</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="1">
+      <text>
+        <t>(Required) The unit of measurement used to specify the source storage duration
+value. Example: hour</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="1">
+      <text>
+        <t>The length of time since the acquisition instrument was last serviced or
+calibrated. This provides a metric for assessing drift in data capture. Example:
+10</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="1">
+      <text>
+        <t>The unit of measurement used to specify the time since acquisition instrument
+calibration value. Example: month</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="1">
       <text>
         <t>(Required) The name of the file containing the ORCID IDs for all contributors to
 this dataset. Example: ./contributors.csv</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="1">
+    <comment ref="N1" authorId="1">
       <text>
         <t>(Required) The top-level directory containing the raw and/or processed data. For
 a single dataset upload, this might be represented as ".", whereas for a data
@@ -79,7 +144,7 @@
 an internal metadata field used solely for data ingestion. Example: ./TEST001-RK</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="1">
+    <comment ref="O1" authorId="1">
       <text>
         <t>(Required) The mapped area value, which refers to the specific area covered or
 captured in various assays. For Visium, it is the area of spots covered by
@@ -92,52 +157,52 @@
 42.25</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="1">
+    <comment ref="P1" authorId="1">
       <text>
         <t>(Required) The unit of measurement for the mapped area value. If mapping area is
 not specified, this field may be left blank. Example: um^2</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="1">
+    <comment ref="Q1" authorId="1">
       <text>
         <t>The capture area on the slide that was used during the process. For example, in
 the case for Visium, this would correspond to areas such as [A1, B1, C1, D1],
 while for HiFi, it would refer to the lane on the flowcell. Example: A1</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="1">
+    <comment ref="R1" authorId="1">
       <text>
         <t>(Required) The width of RNA capture area. Example: 10</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="1">
+    <comment ref="S1" authorId="1">
       <text>
         <t>(Required) The unit of measurement for the capture area width value. If the
 width value is not specified, this field may be left blank. Example: mm</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="1">
+    <comment ref="T1" authorId="1">
       <text>
         <t>(Required) The height of RNA capture area. Example: 10</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="1">
+    <comment ref="U1" authorId="1">
       <text>
         <t>(Required) The unit of measurement for the capture area height value. If the
 height value is not specified, this field may be left blank. Example: mm</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="1">
+    <comment ref="V1" authorId="1">
       <text>
         <t>Permeabilization time used for this tissue section.</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="1">
+    <comment ref="W1" authorId="1">
       <text>
         <t>The unit for the permeabilization time.</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="1">
+    <comment ref="X1" authorId="1">
       <text>
         <t>The company that manufactures the instrument used to prepare the sample (e.g.,
 for staining or other processing steps) prior to the assay. If the instrument
@@ -145,7 +210,7 @@
 preparation occurred, enter "Not applicable". Example: 10X Genomics</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="1">
+    <comment ref="Y1" authorId="1">
       <text>
         <t>The specific model of the instrument used for sample preparation, such as
 staining. Manufacturers may offer multiple models with varying features or
@@ -154,19 +219,19 @@
 applicable". Example: Chromium X</t>
       </text>
     </comment>
-    <comment ref="R1" authorId="1">
+    <comment ref="Z1" authorId="1">
       <text>
         <t>(Required) The segmentation method used to divide the capture are into smaller,
 defined regions for analysis. Example: Cell segmentation</t>
       </text>
     </comment>
-    <comment ref="S1" authorId="1">
+    <comment ref="AA1" authorId="1">
       <text>
         <t>The size (in µm) of each discrete spatial unit ("bin") used to partition the
 capture area in bin-based spatial discretization. Example: 100</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="1">
+    <comment ref="AB1" authorId="1">
       <text>
         <t>(Required) The unique string identifier for the metadata specification version,
 which is easily interpretable by computers for purposes of data validation and
@@ -178,7 +243,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="489">
   <si>
     <t>parent_sample_id</t>
   </si>
@@ -528,6 +593,879 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000448</t>
   </si>
   <si>
+    <t>analyte_class</t>
+  </si>
+  <si>
+    <t>DNA + RNA</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000327</t>
+  </si>
+  <si>
+    <t>Nucleic acid + protein</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000273</t>
+  </si>
+  <si>
+    <t>Chromatin</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C13201</t>
+  </si>
+  <si>
+    <t>Lipid + metabolite + protein</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000478</t>
+  </si>
+  <si>
+    <t>RNA + protein</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000474</t>
+  </si>
+  <si>
+    <t>RNA</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C812</t>
+  </si>
+  <si>
+    <t>Metabolite</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C61154</t>
+  </si>
+  <si>
+    <t>Unsaturated lipid</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000389</t>
+  </si>
+  <si>
+    <t>Lipid + metabolite</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000401</t>
+  </si>
+  <si>
+    <t>Saturated lipid</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000388</t>
+  </si>
+  <si>
+    <t>Lipid</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C616</t>
+  </si>
+  <si>
+    <t>Protein</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17021</t>
+  </si>
+  <si>
+    <t>Fluorochrome</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/CHEBI_51217</t>
+  </si>
+  <si>
+    <t>Collagen</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C16447</t>
+  </si>
+  <si>
+    <t>DNA</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C449</t>
+  </si>
+  <si>
+    <t>Peptide</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C735</t>
+  </si>
+  <si>
+    <t>Polysaccharide</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/CHEBI_18154</t>
+  </si>
+  <si>
+    <t>Endogenous fluorophore</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000131</t>
+  </si>
+  <si>
+    <t>is_targeted</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>acquisition_instrument_vendor</t>
+  </si>
+  <si>
+    <t>BGI Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024848</t>
+  </si>
+  <si>
+    <t>Cytiva</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023581</t>
+  </si>
+  <si>
+    <t>Thermo Fisher Scientific</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008452</t>
+  </si>
+  <si>
+    <t>Zeiss Microscopy</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023607</t>
+  </si>
+  <si>
+    <t>Complete Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027007</t>
+  </si>
+  <si>
+    <t>3DHISTECH</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027042</t>
+  </si>
+  <si>
+    <t>GE Healthcare</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025461</t>
+  </si>
+  <si>
+    <t>Leica Microsystems</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008960</t>
+  </si>
+  <si>
+    <t>Akoya Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023774</t>
+  </si>
+  <si>
+    <t>NanoString</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023912</t>
+  </si>
+  <si>
+    <t>Element Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026453</t>
+  </si>
+  <si>
+    <t>Andor</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023609</t>
+  </si>
+  <si>
+    <t>Huron Digital Pathology</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024996</t>
+  </si>
+  <si>
+    <t>Illumina</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_010233</t>
+  </si>
+  <si>
+    <t>Ionpath</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023605</t>
+  </si>
+  <si>
+    <t>Waters</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024589</t>
+  </si>
+  <si>
+    <t>In-House</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C126386</t>
+  </si>
+  <si>
+    <t>Resolve Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023911</t>
+  </si>
+  <si>
+    <t>Singular Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026683</t>
+  </si>
+  <si>
+    <t>Vizgen</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026274</t>
+  </si>
+  <si>
+    <t>Standard BioTools (Fluidigm)</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023606</t>
+  </si>
+  <si>
+    <t>Sciex</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023651</t>
+  </si>
+  <si>
+    <t>Bruker</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017365</t>
+  </si>
+  <si>
+    <t>Evident Scientific (Olympus)</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024782</t>
+  </si>
+  <si>
+    <t>Keyence</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023604</t>
+  </si>
+  <si>
+    <t>Miltenyi Biotec</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008984</t>
+  </si>
+  <si>
+    <t>Leica Biosystems</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023603</t>
+  </si>
+  <si>
+    <t>Revvity</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027779</t>
+  </si>
+  <si>
+    <t>Cytek Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027071</t>
+  </si>
+  <si>
+    <t>10x Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023672</t>
+  </si>
+  <si>
+    <t>Microscopes International</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027094</t>
+  </si>
+  <si>
+    <t>Hamamatsu</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017105</t>
+  </si>
+  <si>
+    <t>Motic</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024856</t>
+  </si>
+  <si>
+    <t>acquisition_instrument_model</t>
+  </si>
+  <si>
+    <t>SCN400</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023611</t>
+  </si>
+  <si>
+    <t>STELLARIS 5</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024663</t>
+  </si>
+  <si>
+    <t>BZ-X710</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017202</t>
+  </si>
+  <si>
+    <t>Pannoramic MIDI II Digital Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024834</t>
+  </si>
+  <si>
+    <t>Not applicable</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C48660</t>
+  </si>
+  <si>
+    <t>MoticEasyScan One</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024855</t>
+  </si>
+  <si>
+    <t>EVOS M7000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025070</t>
+  </si>
+  <si>
+    <t>NovaSeq X</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024569</t>
+  </si>
+  <si>
+    <t>LSM 710 Confocal Microscope</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_018063</t>
+  </si>
+  <si>
+    <t>NanoZoomer 2.0-HT</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_021658</t>
+  </si>
+  <si>
+    <t>timsTOF Ultra 2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026541</t>
+  </si>
+  <si>
+    <t>Lightsheet 7</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024448</t>
+  </si>
+  <si>
+    <t>Phenocycler-Fusion 1.0</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000316</t>
+  </si>
+  <si>
+    <t>DNBSEQ-T7</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024847</t>
+  </si>
+  <si>
+    <t>timsTOF Pro</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026544</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17998</t>
+  </si>
+  <si>
+    <t>AVITI</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026452</t>
+  </si>
+  <si>
+    <t>DMi8</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026672</t>
+  </si>
+  <si>
+    <t>Opera Phenix Plus HCS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027780</t>
+  </si>
+  <si>
+    <t>timsTOF Pro 2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026545</t>
+  </si>
+  <si>
+    <t>Q Exactive UHMR</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020571</t>
+  </si>
+  <si>
+    <t>Q Exactive</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020565</t>
+  </si>
+  <si>
+    <t>timsTOF SCP</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026542</t>
+  </si>
+  <si>
+    <t>Zyla 4.2 sCMOS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023610</t>
+  </si>
+  <si>
+    <t>Helios</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_019916</t>
+  </si>
+  <si>
+    <t>uScopeHXII-20</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027101</t>
+  </si>
+  <si>
+    <t>Orbitrap Fusion Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020559</t>
+  </si>
+  <si>
+    <t>Custom: Multiphoton</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000317</t>
+  </si>
+  <si>
+    <t>QTRAP 5500</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020517</t>
+  </si>
+  <si>
+    <t>timsTOF Ultra</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026540</t>
+  </si>
+  <si>
+    <t>BZ-X800</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023617</t>
+  </si>
+  <si>
+    <t>CyTOF 2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026551</t>
+  </si>
+  <si>
+    <t>G4X Spatial Sequencer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026684</t>
+  </si>
+  <si>
+    <t>NextSeq 500</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_014983</t>
+  </si>
+  <si>
+    <t>NanoZoomer S360</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023761</t>
+  </si>
+  <si>
+    <t>Hyperion Imaging System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023195</t>
+  </si>
+  <si>
+    <t>NovaSeq X Plus</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024568</t>
+  </si>
+  <si>
+    <t>CyTOF XT</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026344</t>
+  </si>
+  <si>
+    <t>NanoZoomer-SQ</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023763</t>
+  </si>
+  <si>
+    <t>NextSeq 550</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016381</t>
+  </si>
+  <si>
+    <t>Axio Zoom.V16</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027090</t>
+  </si>
+  <si>
+    <t>Digital Spatial Profiler</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_021660</t>
+  </si>
+  <si>
+    <t>timsTOF FleX</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026925</t>
+  </si>
+  <si>
+    <t>timsTOF FleX MALDI-2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023615</t>
+  </si>
+  <si>
+    <t>NanoZoomer S210</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023760</t>
+  </si>
+  <si>
+    <t>BZ-X810</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025160</t>
+  </si>
+  <si>
+    <t>Axio Observer 7</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023694</t>
+  </si>
+  <si>
+    <t>Cytek Northern Lights</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027072</t>
+  </si>
+  <si>
+    <t>Opera Phenix HCS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027817</t>
+  </si>
+  <si>
+    <t>Zeiss LightSheet Z.1</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020919</t>
+  </si>
+  <si>
+    <t>IN Cell Analyzer 2200</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023616</t>
+  </si>
+  <si>
+    <t>timsTOF HT</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026543</t>
+  </si>
+  <si>
+    <t>PhenoImager Fusion</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023274</t>
+  </si>
+  <si>
+    <t>DM6 B</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024857</t>
+  </si>
+  <si>
+    <t>Phenocycler-Fusion 2.0</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023773</t>
+  </si>
+  <si>
+    <t>Aperio CS2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025111</t>
+  </si>
+  <si>
+    <t>Orbitrap Fusion Lumos Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020562</t>
+  </si>
+  <si>
+    <t>Resolve Biosciences Molecular Cartography</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024449</t>
+  </si>
+  <si>
+    <t>MALDI timsTOF Flex Prototype</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000433</t>
+  </si>
+  <si>
+    <t>TissueScope LE Slide Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024995</t>
+  </si>
+  <si>
+    <t>VS200 Slide Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024783</t>
+  </si>
+  <si>
+    <t>Axio Observer 5</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023692</t>
+  </si>
+  <si>
+    <t>NanoZoomer 2.0-RS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_028001</t>
+  </si>
+  <si>
+    <t>Axio Observer 3</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023693</t>
+  </si>
+  <si>
+    <t>HiSeq 2500</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016383</t>
+  </si>
+  <si>
+    <t>Orbitrap Eclipse Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023618</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027323</t>
+  </si>
+  <si>
+    <t>MERSCOPE</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000404</t>
+  </si>
+  <si>
+    <t>NextSeq 2000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023614</t>
+  </si>
+  <si>
+    <t>NovaSeq 6000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016387</t>
+  </si>
+  <si>
+    <t>HiSeq 4000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016386</t>
+  </si>
+  <si>
+    <t>solariX</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027095</t>
+  </si>
+  <si>
+    <t>Panoramic 150 Digital Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027467</t>
+  </si>
+  <si>
+    <t>Aperio AT2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_021256</t>
+  </si>
+  <si>
+    <t>MIBIscope</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023613</t>
+  </si>
+  <si>
+    <t>SYNAPT G2-Si</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027782</t>
+  </si>
+  <si>
+    <t>MACSima System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027923</t>
+  </si>
+  <si>
+    <t>Biomark HD</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_022658</t>
+  </si>
+  <si>
+    <t>NanoZoomer S60</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023762</t>
+  </si>
+  <si>
+    <t>CosMx Spatial Molecular Imager</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023909</t>
+  </si>
+  <si>
+    <t>MERSCOPE Ultra</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026273</t>
+  </si>
+  <si>
+    <t>Axio Scan.Z1</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020927</t>
+  </si>
+  <si>
+    <t>Juno System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027198</t>
+  </si>
+  <si>
+    <t>Q Exactive HF</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020558</t>
+  </si>
+  <si>
+    <t>Xenium Analyzer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023910</t>
+  </si>
+  <si>
+    <t>source_storage_duration_value</t>
+  </si>
+  <si>
+    <t>source_storage_duration_unit</t>
+  </si>
+  <si>
+    <t>hour</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000032</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000035</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000036</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000033</t>
+  </si>
+  <si>
+    <t>minute</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000031</t>
+  </si>
+  <si>
+    <t>time_since_acquisition_instrument_calibration_value</t>
+  </si>
+  <si>
+    <t>time_since_acquisition_instrument_calibration_unit</t>
+  </si>
+  <si>
     <t>contributors_path</t>
   </si>
   <si>
@@ -615,39 +1553,9 @@
     <t>permeabilization_time_unit</t>
   </si>
   <si>
-    <t>minute</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000031</t>
-  </si>
-  <si>
     <t>preparation_instrument_vendor</t>
   </si>
   <si>
-    <t>In-House</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C126386</t>
-  </si>
-  <si>
-    <t>Leica Biosystems</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023603</t>
-  </si>
-  <si>
-    <t>Not applicable</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C48660</t>
-  </si>
-  <si>
-    <t>Thermo Fisher Scientific</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_008452</t>
-  </si>
-  <si>
     <t>Roche Diagnostics</t>
   </si>
   <si>
@@ -660,30 +1568,6 @@
     <t>https://identifiers.org/RRID:SCR_023734</t>
   </si>
   <si>
-    <t>10x Genomics</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023672</t>
-  </si>
-  <si>
-    <t>Hamamatsu</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_017105</t>
-  </si>
-  <si>
-    <t>Ionpath</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023605</t>
-  </si>
-  <si>
-    <t>Akoya Biosciences</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023774</t>
-  </si>
-  <si>
     <t>SunChrom</t>
   </si>
   <si>
@@ -693,24 +1577,12 @@
     <t>preparation_instrument_model</t>
   </si>
   <si>
-    <t>NanoZoomer S210</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023760</t>
-  </si>
-  <si>
     <t>Sublimator</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_023729</t>
   </si>
   <si>
-    <t>EVOS M7000</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025070</t>
-  </si>
-  <si>
     <t>Chromium Controller</t>
   </si>
   <si>
@@ -723,18 +1595,6 @@
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65167</t>
   </si>
   <si>
-    <t>NanoZoomer S360</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023761</t>
-  </si>
-  <si>
-    <t>NanoZoomer S60</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023762</t>
-  </si>
-  <si>
     <t>Chromium X</t>
   </si>
   <si>
@@ -843,7 +1703,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2026-03-27T11:11:56-07:00</t>
+    <t>2026-04-06T18:05:20-07:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -902,7 +1762,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyAlignment="true" applyFill="true">
       <alignment horizontal="center"/>
@@ -910,6 +1770,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -937,29 +1805,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" style="2" width="14.39453125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" style="3" width="5.46875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" style="4" width="20.234375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" style="5" width="10.59765625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" style="6" width="14.5859375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" style="7" width="8.46484375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" style="8" width="15.984375" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" style="9" width="14.984375" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" style="10" width="12.98828125" customWidth="true" bestFit="true"/>
-    <col min="10" max="10" style="11" width="20.58203125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" style="12" width="19.58203125" customWidth="true" bestFit="true"/>
-    <col min="12" max="12" style="13" width="21.21875" customWidth="true" bestFit="true"/>
-    <col min="13" max="13" style="14" width="20.21875" customWidth="true" bestFit="true"/>
-    <col min="14" max="14" style="15" width="22.80078125" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" style="16" width="21.80078125" customWidth="true" bestFit="true"/>
-    <col min="16" max="16" style="17" width="25.0859375" customWidth="true" bestFit="true"/>
-    <col min="17" max="17" style="18" width="24.57421875" customWidth="true" bestFit="true"/>
-    <col min="18" max="18" style="19" width="24.734375" customWidth="true" bestFit="true"/>
-    <col min="19" max="19" style="20" width="7.17578125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" style="21" width="16.91796875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" style="6" width="10.9296875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" style="7" width="9.40234375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" style="8" width="24.5546875" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" style="9" width="24.0390625" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" style="10" width="24.63671875" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" style="11" width="23.63671875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" style="12" width="41.1015625" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" style="13" width="40.1015625" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" style="14" width="14.5859375" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" style="15" width="8.46484375" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" style="16" width="15.984375" customWidth="true" bestFit="true"/>
+    <col min="16" max="16" style="17" width="14.984375" customWidth="true" bestFit="true"/>
+    <col min="17" max="17" style="18" width="12.98828125" customWidth="true" bestFit="true"/>
+    <col min="18" max="18" style="19" width="20.58203125" customWidth="true" bestFit="true"/>
+    <col min="19" max="19" style="20" width="19.58203125" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" style="21" width="21.21875" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" style="22" width="20.21875" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" style="23" width="22.80078125" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" style="24" width="21.80078125" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" style="25" width="25.0859375" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" style="26" width="24.57421875" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" style="27" width="24.734375" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" style="28" width="7.17578125" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" style="29" width="16.91796875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -979,102 +1855,152 @@
         <v>116</v>
       </c>
       <c r="F1" t="s" s="1">
-        <v>117</v>
+        <v>153</v>
       </c>
       <c r="G1" t="s" s="1">
-        <v>118</v>
+        <v>156</v>
       </c>
       <c r="H1" t="s" s="1">
-        <v>119</v>
+        <v>223</v>
       </c>
       <c r="I1" t="s" s="1">
-        <v>124</v>
+        <v>393</v>
       </c>
       <c r="J1" t="s" s="1">
-        <v>137</v>
+        <v>394</v>
       </c>
       <c r="K1" t="s" s="1">
-        <v>138</v>
+        <v>405</v>
       </c>
       <c r="L1" t="s" s="1">
-        <v>141</v>
+        <v>406</v>
       </c>
       <c r="M1" t="s" s="1">
-        <v>142</v>
+        <v>407</v>
       </c>
       <c r="N1" t="s" s="1">
-        <v>143</v>
+        <v>408</v>
       </c>
       <c r="O1" t="s" s="1">
-        <v>144</v>
+        <v>409</v>
       </c>
       <c r="P1" t="s" s="1">
-        <v>147</v>
+        <v>410</v>
       </c>
       <c r="Q1" t="s" s="1">
-        <v>170</v>
+        <v>415</v>
       </c>
       <c r="R1" t="s" s="1">
-        <v>207</v>
+        <v>428</v>
       </c>
       <c r="S1" t="s" s="1">
-        <v>214</v>
+        <v>429</v>
       </c>
       <c r="T1" t="s" s="1">
-        <v>215</v>
+        <v>432</v>
+      </c>
+      <c r="U1" t="s" s="1">
+        <v>433</v>
+      </c>
+      <c r="V1" t="s" s="1">
+        <v>434</v>
+      </c>
+      <c r="W1" t="s" s="1">
+        <v>435</v>
+      </c>
+      <c r="X1" t="s" s="1">
+        <v>436</v>
+      </c>
+      <c r="Y1" t="s" s="1">
+        <v>443</v>
+      </c>
+      <c r="Z1" t="s" s="1">
+        <v>472</v>
+      </c>
+      <c r="AA1" t="s" s="1">
+        <v>479</v>
+      </c>
+      <c r="AB1" t="s" s="1">
+        <v>480</v>
       </c>
     </row>
     <row r="2">
       <c r="D2" t="s" s="5">
         <v>62</v>
       </c>
-      <c r="T2" t="s" s="21">
-        <v>216</v>
+      <c r="AB2" t="s" s="29">
+        <v>481</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="13">
+  <dataValidations count="21">
     <dataValidation type="list" sqref="D2:D1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'dataset_type'!$A$1:$A$56</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" sqref="G2:G1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="list" sqref="E2:E1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'analyte_class'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="F2:F1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'is_targeted'!$A$1:$A$2</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="G2:G1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'acquisition_instrument_vendor'!$A$1:$A$33</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="H2:H1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'acquisition_instrument_model'!$A$1:$A$86</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="I2:I1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
+      <formula1>0</formula1>
+      <formula2/>
+    </dataValidation>
+    <dataValidation type="list" sqref="J2:J1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'source_storage_duration_unit'!$A$1:$A$5</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="K2:K1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
+      <formula1>0</formula1>
+      <formula2/>
+    </dataValidation>
+    <dataValidation type="list" sqref="L2:L1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+      <formula1>'time_since_acquisition_instrume'!$A$1:$A$3</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" sqref="O2:O1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-3.4028235E38</formula1>
       <formula2>3.4028235E38</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="H2:H1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="P2:P1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'mapped_area_unit'!$A$1:$A$2</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="I2:I1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="Q2:Q1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'capture_area_id'!$A$1:$A$12</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="J2:J1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="R2:R1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
       <formula1>0</formula1>
       <formula2/>
     </dataValidation>
-    <dataValidation type="list" sqref="K2:K1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="S2:S1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'capture_area_width_unit'!$A$1:$A$1</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="L2:L1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="T2:T1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
       <formula1>0</formula1>
       <formula2/>
     </dataValidation>
-    <dataValidation type="list" sqref="M2:M1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="U2:U1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'capture_area_height_unit'!$A$1:$A$1</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="between" sqref="N2:N1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
+    <dataValidation type="whole" operator="between" sqref="V2:V1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-2147483648</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="O2:O1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="W2:W1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'permeabilization_time_unit'!$A$1:$A$1</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="P2:P1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="X2:X1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'preparation_instrument_vendor'!$A$1:$A$11</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:Q1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="Y2:Y1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'preparation_instrument_model'!$A$1:$A$19</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="R2:R1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
+    <dataValidation type="list" sqref="Z2:Z1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'spatial_discreatization_method'!$A$1:$A$3</formula1>
     </dataValidation>
   </dataValidations>
@@ -1086,31 +2012,67 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>208</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>209</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>210</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>211</v>
+        <v>417</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>212</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>213</v>
+        <v>418</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>427</v>
       </c>
     </row>
   </sheetData>
@@ -1119,6 +2081,354 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>430</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>431</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>430</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>431</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>403</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>404</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>185</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>442</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>444</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>446</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>448</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>292</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>379</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>450</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>452</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>454</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>456</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>458</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>460</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>462</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>464</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>466</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>468</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>470</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>471</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>473</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>475</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>477</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>478</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1131,16 +2441,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>217</v>
+        <v>482</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>218</v>
+        <v>483</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>220</v>
+        <v>485</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>222</v>
+        <v>487</v>
       </c>
     </row>
     <row r="2">
@@ -1148,13 +2458,13 @@
         <v>62</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>219</v>
+        <v>484</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>221</v>
+        <v>486</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>223</v>
+        <v>488</v>
       </c>
     </row>
   </sheetData>
@@ -1622,23 +2932,151 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>121</v>
+      </c>
+      <c r="B3" t="s" s="0">
         <v>122</v>
       </c>
-      <c r="B2" t="s" s="0">
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
         <v>123</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>125</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>135</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>137</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>139</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>145</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>147</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>149</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>151</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -1648,67 +3086,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>125</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>136</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -1718,15 +3106,271 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>140</v>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>163</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>165</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>169</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>171</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>181</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>183</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>185</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>187</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>193</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>195</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>213</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -1736,15 +3380,695 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B86"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>139</v>
+        <v>224</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>140</v>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>226</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>234</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>238</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>240</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>242</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>248</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>254</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>268</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>270</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>272</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>274</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>276</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>286</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>288</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>290</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>292</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>294</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="0">
+        <v>296</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>300</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="0">
+        <v>304</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="0">
+        <v>314</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="0">
+        <v>320</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>322</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>324</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>326</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>328</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B56" t="s" s="0">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="B57" t="s" s="0">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>338</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>340</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="0">
+        <v>342</v>
+      </c>
+      <c r="B60" t="s" s="0">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="0">
+        <v>344</v>
+      </c>
+      <c r="B61" t="s" s="0">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="0">
+        <v>346</v>
+      </c>
+      <c r="B62" t="s" s="0">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="0">
+        <v>348</v>
+      </c>
+      <c r="B63" t="s" s="0">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="0">
+        <v>350</v>
+      </c>
+      <c r="B64" t="s" s="0">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="0">
+        <v>352</v>
+      </c>
+      <c r="B65" t="s" s="0">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="B66" t="s" s="0">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="B67" t="s" s="0">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="B68" t="s" s="0">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="B69" t="s" s="0">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s" s="0">
+        <v>361</v>
+      </c>
+      <c r="B70" t="s" s="0">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B71" t="s" s="0">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s" s="0">
+        <v>363</v>
+      </c>
+      <c r="B72" t="s" s="0">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s" s="0">
+        <v>365</v>
+      </c>
+      <c r="B73" t="s" s="0">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s" s="0">
+        <v>367</v>
+      </c>
+      <c r="B74" t="s" s="0">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s" s="0">
+        <v>369</v>
+      </c>
+      <c r="B75" t="s" s="0">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s" s="0">
+        <v>371</v>
+      </c>
+      <c r="B76" t="s" s="0">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s" s="0">
+        <v>373</v>
+      </c>
+      <c r="B77" t="s" s="0">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s" s="0">
+        <v>375</v>
+      </c>
+      <c r="B78" t="s" s="0">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s" s="0">
+        <v>377</v>
+      </c>
+      <c r="B79" t="s" s="0">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s" s="0">
+        <v>379</v>
+      </c>
+      <c r="B80" t="s" s="0">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s" s="0">
+        <v>381</v>
+      </c>
+      <c r="B81" t="s" s="0">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s" s="0">
+        <v>383</v>
+      </c>
+      <c r="B82" t="s" s="0">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s" s="0">
+        <v>385</v>
+      </c>
+      <c r="B83" t="s" s="0">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s" s="0">
+        <v>387</v>
+      </c>
+      <c r="B84" t="s" s="0">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s" s="0">
+        <v>389</v>
+      </c>
+      <c r="B85" t="s" s="0">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s" s="0">
+        <v>391</v>
+      </c>
+      <c r="B86" t="s" s="0">
+        <v>392</v>
       </c>
     </row>
   </sheetData>
@@ -1754,15 +4078,47 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>145</v>
+        <v>395</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>146</v>
+        <v>396</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>397</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>399</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>401</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>403</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>404</v>
       </c>
     </row>
   </sheetData>
@@ -1772,95 +4128,31 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>148</v>
+        <v>397</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>149</v>
+        <v>398</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>150</v>
+        <v>399</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>151</v>
+        <v>400</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>152</v>
+        <v>401</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>154</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>156</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>158</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>160</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>162</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="B9" t="s" s="0">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>166</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>168</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>169</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -1870,159 +4162,23 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>171</v>
+        <v>411</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>172</v>
+        <v>412</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>152</v>
+        <v>413</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>173</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>175</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>177</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>179</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>181</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>183</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>185</v>
-      </c>
-      <c r="B9" t="s" s="0">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>187</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>189</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>191</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="0">
-        <v>193</v>
-      </c>
-      <c r="B13" t="s" s="0">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="0">
-        <v>195</v>
-      </c>
-      <c r="B14" t="s" s="0">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="0">
-        <v>197</v>
-      </c>
-      <c r="B15" t="s" s="0">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>199</v>
-      </c>
-      <c r="B16" t="s" s="0">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s" s="0">
-        <v>201</v>
-      </c>
-      <c r="B17" t="s" s="0">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>203</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>205</v>
-      </c>
-      <c r="B19" t="s" s="0">
-        <v>206</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>